<commit_message>
Aggiornato resa.xlsx da lbianco via Streamlit
</commit_message>
<xml_diff>
--- a/resa.xlsx
+++ b/resa.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3741" uniqueCount="880">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3870" uniqueCount="907">
   <si>
     <t>Codice</t>
   </si>
@@ -2657,6 +2657,87 @@
   </si>
   <si>
     <t>PERM.RTG-ISDN-VDSL</t>
+  </si>
+  <si>
+    <t>ADSL1005610179</t>
+  </si>
+  <si>
+    <t>98209608</t>
+  </si>
+  <si>
+    <t>VIA LUIGI CASSIA 53/B</t>
+  </si>
+  <si>
+    <t>DTU0070808755</t>
+  </si>
+  <si>
+    <t>93114750489</t>
+  </si>
+  <si>
+    <t>E80098209608</t>
+  </si>
+  <si>
+    <t>30/03/2026 11:22</t>
+  </si>
+  <si>
+    <t>MTW25182SA</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>B43341803</t>
+  </si>
+  <si>
+    <t>ADSL1005672491</t>
+  </si>
+  <si>
+    <t>98626054</t>
+  </si>
+  <si>
+    <t>VIA LE FORNACI 91</t>
+  </si>
+  <si>
+    <t>DTU0071125605</t>
+  </si>
+  <si>
+    <t>93114762017</t>
+  </si>
+  <si>
+    <t>E80098626054</t>
+  </si>
+  <si>
+    <t>15/04/2026 14:50</t>
+  </si>
+  <si>
+    <t>B43752702</t>
+  </si>
+  <si>
+    <t>ADSL1005688660</t>
+  </si>
+  <si>
+    <t>98734674</t>
+  </si>
+  <si>
+    <t>VIA MARESCIALLO DELL'ALI 16</t>
+  </si>
+  <si>
+    <t>DTU0071065689</t>
+  </si>
+  <si>
+    <t>0931452521</t>
+  </si>
+  <si>
+    <t>E80098734674</t>
+  </si>
+  <si>
+    <t>20/04/2026 12:40</t>
+  </si>
+  <si>
+    <t>98505734</t>
+  </si>
+  <si>
+    <t>B43863823</t>
   </si>
 </sst>
 </file>
@@ -2993,7 +3074,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AQ87"/>
+  <dimension ref="A1:AQ90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1" customWidth="1"/>
@@ -14397,6 +14478,399 @@
         <v>622</v>
       </c>
     </row>
+    <row r="88" spans="1:43">
+      <c r="A88" s="1" t="s">
+        <v>880</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>881</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H88" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I88" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="J88" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="K88" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L88" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="M88" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="N88" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="O88" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="P88" s="1" t="s">
+        <v>882</v>
+      </c>
+      <c r="Q88" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="R88" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="S88" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="T88" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="U88" s="1" t="s">
+        <v>883</v>
+      </c>
+      <c r="V88" s="1" t="s">
+        <v>884</v>
+      </c>
+      <c r="W88" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="X88" s="1" t="s">
+        <v>885</v>
+      </c>
+      <c r="Y88" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z88" s="1" t="s">
+        <v>886</v>
+      </c>
+      <c r="AA88" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="AB88" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="AC88" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD88" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AE88" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="AF88" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AG88" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="AH88" s="1" t="s">
+        <v>887</v>
+      </c>
+      <c r="AI88" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AJ88" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AK88" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="AL88" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM88" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="AN88" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AO88" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AP88" s="1" t="s">
+        <v>888</v>
+      </c>
+      <c r="AQ88" s="1" t="s">
+        <v>889</v>
+      </c>
+    </row>
+    <row r="89" spans="1:43">
+      <c r="A89" s="1" t="s">
+        <v>890</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>891</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H89" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I89" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="J89" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="K89" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L89" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M89" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="N89" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="O89" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="P89" s="1" t="s">
+        <v>892</v>
+      </c>
+      <c r="Q89" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="R89" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="S89" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="T89" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="U89" s="1" t="s">
+        <v>893</v>
+      </c>
+      <c r="V89" s="1" t="s">
+        <v>894</v>
+      </c>
+      <c r="W89" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="X89" s="1" t="s">
+        <v>895</v>
+      </c>
+      <c r="Y89" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z89" s="1" t="s">
+        <v>896</v>
+      </c>
+      <c r="AA89" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB89" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AC89" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD89" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AE89" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="AF89" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AG89" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="AH89" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="AI89" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AJ89" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AK89" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="AL89" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM89" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="AN89" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AO89" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AP89" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="AQ89" s="1" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="90" spans="1:43">
+      <c r="A90" s="1" t="s">
+        <v>898</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>899</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H90" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I90" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="J90" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="K90" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="L90" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="M90" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="N90" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="O90" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="P90" s="1" t="s">
+        <v>900</v>
+      </c>
+      <c r="Q90" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="R90" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="S90" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="T90" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="U90" s="1" t="s">
+        <v>901</v>
+      </c>
+      <c r="V90" s="1" t="s">
+        <v>902</v>
+      </c>
+      <c r="W90" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="X90" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="Y90" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="Z90" s="1" t="s">
+        <v>904</v>
+      </c>
+      <c r="AA90" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="AB90" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="AC90" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD90" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AE90" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF90" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AG90" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="AH90" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI90" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="AJ90" s="1" t="s">
+        <v>905</v>
+      </c>
+      <c r="AK90" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="AL90" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM90" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="AN90" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AO90" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AP90" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="AQ90" s="1" t="s">
+        <v>906</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AQ76"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>